<commit_message>
feat: complete Quality Education platform ready for 24/7 cloud deployment
</commit_message>
<xml_diff>
--- a/students_records.xlsx
+++ b/students_records.xlsx
@@ -397,17 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:G13"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="30.83203125" customWidth="1"/>
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="32.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,13 +428,7 @@
         <v>Contact Number</v>
       </c>
       <c r="G1" t="str">
-        <v>Class/Course</v>
-      </c>
-      <c r="H1" t="str">
         <v>Enrollment Date</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Registration Timestamp</v>
       </c>
     </row>
     <row r="2">
@@ -459,13 +451,7 @@
         <v>+91 98765 43210</v>
       </c>
       <c r="G2" t="str">
-        <v>Computer Science &amp; AI</v>
-      </c>
-      <c r="H2" t="str">
         <v>2026-01-15</v>
-      </c>
-      <c r="I2" t="str">
-        <v>2026-09-27 06:05:32</v>
       </c>
     </row>
     <row r="3">
@@ -488,13 +474,7 @@
         <v>+91 98123 45678</v>
       </c>
       <c r="G3" t="str">
-        <v>Environmental Science &amp; Sustainability</v>
-      </c>
-      <c r="H3" t="str">
         <v>2026-02-01</v>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-09-27 06:05:32</v>
       </c>
     </row>
     <row r="4">
@@ -517,13 +497,7 @@
         <v>+91 97654 32109</v>
       </c>
       <c r="G4" t="str">
-        <v>Advanced Mathematics &amp; Statistics</v>
-      </c>
-      <c r="H4" t="str">
         <v>2026-02-14</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-09-27 06:05:32</v>
       </c>
     </row>
     <row r="5">
@@ -546,13 +520,7 @@
         <v>+91 98451 23456</v>
       </c>
       <c r="G5" t="str">
-        <v>Global Literature &amp; Communication</v>
-      </c>
-      <c r="H5" t="str">
         <v>2026-03-01</v>
-      </c>
-      <c r="I5" t="str">
-        <v>2026-09-27 06:05:32</v>
       </c>
     </row>
     <row r="6">
@@ -575,13 +543,7 @@
         <v>+91 99012 34567</v>
       </c>
       <c r="G6" t="str">
-        <v>Business Ethics &amp; Leadership</v>
-      </c>
-      <c r="H6" t="str">
         <v>2026-03-10</v>
-      </c>
-      <c r="I6" t="str">
-        <v>2026-09-27 06:05:32</v>
       </c>
     </row>
     <row r="7">
@@ -604,13 +566,7 @@
         <v>+91 98220 12345</v>
       </c>
       <c r="G7" t="str">
-        <v>Computer Science &amp; AI</v>
-      </c>
-      <c r="H7" t="str">
         <v>2026-09-27</v>
-      </c>
-      <c r="I7" t="str">
-        <v>2026-09-27 06:05:47</v>
       </c>
     </row>
     <row r="8">
@@ -633,13 +589,7 @@
         <v>+91 98331 45678</v>
       </c>
       <c r="G8" t="str">
-        <v>Environmental Science &amp; Sustainability</v>
-      </c>
-      <c r="H8" t="str">
         <v>2026-09-27</v>
-      </c>
-      <c r="I8" t="str">
-        <v>2026-09-27 06:15:02</v>
       </c>
     </row>
     <row r="9">
@@ -662,18 +612,104 @@
         <v>+91 98990 12345</v>
       </c>
       <c r="G9" t="str">
-        <v>Computer Science &amp; AI</v>
-      </c>
-      <c r="H9" t="str">
         <v>2026-09-27</v>
       </c>
-      <c r="I9" t="str">
-        <v>2026-09-27 06:26:49</v>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>240760107084</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Kanani Het Girishbhai</v>
+      </c>
+      <c r="C10">
+        <v>19</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E10" t="str">
+        <v>hetkanani8302@gmail.com</v>
+      </c>
+      <c r="F10" t="str">
+        <v>9327410137</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>240760107053</v>
+      </c>
+      <c r="B11" t="str">
+        <v>SRUSHTI GHANSHYAM GHORI</v>
+      </c>
+      <c r="C11">
+        <v>20</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E11" t="str">
+        <v>srushtighori07@gmail.com</v>
+      </c>
+      <c r="F11" t="str">
+        <v>8780663905</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-27</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>STU-TEST-999</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Priya Sharma</v>
+      </c>
+      <c r="C12">
+        <v>21</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Female</v>
+      </c>
+      <c r="E12" t="str">
+        <v>priya.sharma@example.com</v>
+      </c>
+      <c r="F12" t="str">
+        <v>+91 9876543210</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>STU-LIVE-001</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Vikram Aditya</v>
+      </c>
+      <c r="C13">
+        <v>23</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Male</v>
+      </c>
+      <c r="E13" t="str">
+        <v>vikram.aditya@example.com</v>
+      </c>
+      <c r="F13" t="str">
+        <v>+91 9812345678</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-27</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>